<commit_message>
day 9 - two pair sum using 2 pointer
</commit_message>
<xml_diff>
--- a/3aed9d04-2385-4fdd-b403-316e5db325c7.xlsx
+++ b/3aed9d04-2385-4fdd-b403-316e5db325c7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{89501D03-1FDF-4C21-8EB1-59F56B47B372}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B982B9D-4C91-497D-B8DB-7E29F7FB531E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,6 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'130-Day Plan'!$A$1:$J$131</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -1415,7 +1414,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:J131"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1547,7 +1545,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1766,7 +1764,7 @@
         <v>37</v>
       </c>
       <c r="H12" s="7" t="s">
-        <v>15</v>
+        <v>302</v>
       </c>
       <c r="I12" s="3"/>
       <c r="J12" s="7"/>
@@ -1794,12 +1792,12 @@
         <v>39</v>
       </c>
       <c r="H13" s="7" t="s">
-        <v>15</v>
+        <v>302</v>
       </c>
       <c r="I13" s="3"/>
       <c r="J13" s="7"/>
     </row>
-    <row r="14" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1883,7 +1881,7 @@
       <c r="I16" s="3"/>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1911,7 +1909,7 @@
       <c r="I17" s="3"/>
       <c r="J17" s="7"/>
     </row>
-    <row r="18" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1939,7 +1937,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="7"/>
     </row>
-    <row r="19" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1995,7 +1993,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="7"/>
     </row>
-    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2023,7 +2021,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="7"/>
     </row>
-    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2051,7 +2049,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="7"/>
     </row>
-    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2079,7 +2077,7 @@
       <c r="I23" s="3"/>
       <c r="J23" s="7"/>
     </row>
-    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2107,7 +2105,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="7"/>
     </row>
-    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2135,7 +2133,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="7"/>
     </row>
-    <row r="26" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2163,7 +2161,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="7"/>
     </row>
-    <row r="27" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2219,7 +2217,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="7"/>
     </row>
-    <row r="29" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2247,7 +2245,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="7"/>
     </row>
-    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2275,7 +2273,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="7"/>
     </row>
-    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2303,7 +2301,7 @@
       <c r="I31" s="3"/>
       <c r="J31" s="7"/>
     </row>
-    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2499,7 +2497,7 @@
       <c r="I38" s="3"/>
       <c r="J38" s="7"/>
     </row>
-    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2527,7 +2525,7 @@
       <c r="I39" s="3"/>
       <c r="J39" s="7"/>
     </row>
-    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2583,7 +2581,7 @@
       <c r="I41" s="3"/>
       <c r="J41" s="7"/>
     </row>
-    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2611,7 +2609,7 @@
       <c r="I42" s="3"/>
       <c r="J42" s="7"/>
     </row>
-    <row r="43" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2807,7 +2805,7 @@
       <c r="I49" s="3"/>
       <c r="J49" s="7"/>
     </row>
-    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2835,7 +2833,7 @@
       <c r="I50" s="3"/>
       <c r="J50" s="7"/>
     </row>
-    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2863,7 +2861,7 @@
       <c r="I51" s="3"/>
       <c r="J51" s="7"/>
     </row>
-    <row r="52" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2891,7 +2889,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="7"/>
     </row>
-    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2919,7 +2917,7 @@
       <c r="I53" s="3"/>
       <c r="J53" s="7"/>
     </row>
-    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -3003,7 +3001,7 @@
       <c r="I56" s="3"/>
       <c r="J56" s="7"/>
     </row>
-    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -3031,7 +3029,7 @@
       <c r="I57" s="3"/>
       <c r="J57" s="7"/>
     </row>
-    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3087,7 +3085,7 @@
       <c r="I59" s="3"/>
       <c r="J59" s="7"/>
     </row>
-    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3115,7 +3113,7 @@
       <c r="I60" s="3"/>
       <c r="J60" s="7"/>
     </row>
-    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -3227,7 +3225,7 @@
       <c r="I64" s="3"/>
       <c r="J64" s="7"/>
     </row>
-    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -3255,7 +3253,7 @@
       <c r="I65" s="3"/>
       <c r="J65" s="7"/>
     </row>
-    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -3283,7 +3281,7 @@
       <c r="I66" s="3"/>
       <c r="J66" s="7"/>
     </row>
-    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -3311,7 +3309,7 @@
       <c r="I67" s="3"/>
       <c r="J67" s="7"/>
     </row>
-    <row r="68" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -3339,7 +3337,7 @@
       <c r="I68" s="3"/>
       <c r="J68" s="7"/>
     </row>
-    <row r="69" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3479,7 +3477,7 @@
       <c r="I73" s="3"/>
       <c r="J73" s="7"/>
     </row>
-    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3591,7 +3589,7 @@
       <c r="I77" s="3"/>
       <c r="J77" s="7"/>
     </row>
-    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3619,7 +3617,7 @@
       <c r="I78" s="3"/>
       <c r="J78" s="7"/>
     </row>
-    <row r="79" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3647,7 +3645,7 @@
       <c r="I79" s="3"/>
       <c r="J79" s="7"/>
     </row>
-    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3675,7 +3673,7 @@
       <c r="I80" s="3"/>
       <c r="J80" s="7"/>
     </row>
-    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3703,7 +3701,7 @@
       <c r="I81" s="3"/>
       <c r="J81" s="7"/>
     </row>
-    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -3759,7 +3757,7 @@
       <c r="I83" s="3"/>
       <c r="J83" s="7"/>
     </row>
-    <row r="84" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -3787,7 +3785,7 @@
       <c r="I84" s="3"/>
       <c r="J84" s="7"/>
     </row>
-    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3815,7 +3813,7 @@
       <c r="I85" s="3"/>
       <c r="J85" s="7"/>
     </row>
-    <row r="86" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3843,7 +3841,7 @@
       <c r="I86" s="3"/>
       <c r="J86" s="7"/>
     </row>
-    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3871,7 +3869,7 @@
       <c r="I87" s="3"/>
       <c r="J87" s="7"/>
     </row>
-    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3899,7 +3897,7 @@
       <c r="I88" s="3"/>
       <c r="J88" s="7"/>
     </row>
-    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3927,7 +3925,7 @@
       <c r="I89" s="3"/>
       <c r="J89" s="7"/>
     </row>
-    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3955,7 +3953,7 @@
       <c r="I90" s="3"/>
       <c r="J90" s="7"/>
     </row>
-    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3983,7 +3981,7 @@
       <c r="I91" s="3"/>
       <c r="J91" s="7"/>
     </row>
-    <row r="92" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -4011,7 +4009,7 @@
       <c r="I92" s="3"/>
       <c r="J92" s="7"/>
     </row>
-    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -4039,7 +4037,7 @@
       <c r="I93" s="3"/>
       <c r="J93" s="7"/>
     </row>
-    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -4067,7 +4065,7 @@
       <c r="I94" s="3"/>
       <c r="J94" s="7"/>
     </row>
-    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -4095,7 +4093,7 @@
       <c r="I95" s="3"/>
       <c r="J95" s="7"/>
     </row>
-    <row r="96" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -4123,7 +4121,7 @@
       <c r="I96" s="3"/>
       <c r="J96" s="7"/>
     </row>
-    <row r="97" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -4151,7 +4149,7 @@
       <c r="I97" s="3"/>
       <c r="J97" s="7"/>
     </row>
-    <row r="98" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -4179,7 +4177,7 @@
       <c r="I98" s="3"/>
       <c r="J98" s="7"/>
     </row>
-    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -4235,7 +4233,7 @@
       <c r="I100" s="3"/>
       <c r="J100" s="7"/>
     </row>
-    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -4263,7 +4261,7 @@
       <c r="I101" s="3"/>
       <c r="J101" s="7"/>
     </row>
-    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -4291,7 +4289,7 @@
       <c r="I102" s="3"/>
       <c r="J102" s="7"/>
     </row>
-    <row r="103" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -4319,7 +4317,7 @@
       <c r="I103" s="3"/>
       <c r="J103" s="7"/>
     </row>
-    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -4347,7 +4345,7 @@
       <c r="I104" s="3"/>
       <c r="J104" s="7"/>
     </row>
-    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -4375,7 +4373,7 @@
       <c r="I105" s="3"/>
       <c r="J105" s="7"/>
     </row>
-    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -4403,7 +4401,7 @@
       <c r="I106" s="3"/>
       <c r="J106" s="7"/>
     </row>
-    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -4431,7 +4429,7 @@
       <c r="I107" s="3"/>
       <c r="J107" s="7"/>
     </row>
-    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -4459,7 +4457,7 @@
       <c r="I108" s="3"/>
       <c r="J108" s="7"/>
     </row>
-    <row r="109" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -4487,7 +4485,7 @@
       <c r="I109" s="3"/>
       <c r="J109" s="7"/>
     </row>
-    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -4515,7 +4513,7 @@
       <c r="I110" s="3"/>
       <c r="J110" s="7"/>
     </row>
-    <row r="111" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -4543,7 +4541,7 @@
       <c r="I111" s="3"/>
       <c r="J111" s="7"/>
     </row>
-    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -4571,7 +4569,7 @@
       <c r="I112" s="3"/>
       <c r="J112" s="7"/>
     </row>
-    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -4599,7 +4597,7 @@
       <c r="I113" s="3"/>
       <c r="J113" s="7"/>
     </row>
-    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -4627,7 +4625,7 @@
       <c r="I114" s="3"/>
       <c r="J114" s="7"/>
     </row>
-    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -4655,7 +4653,7 @@
       <c r="I115" s="3"/>
       <c r="J115" s="7"/>
     </row>
-    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -4683,7 +4681,7 @@
       <c r="I116" s="3"/>
       <c r="J116" s="7"/>
     </row>
-    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -4711,7 +4709,7 @@
       <c r="I117" s="3"/>
       <c r="J117" s="7"/>
     </row>
-    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -4767,7 +4765,7 @@
       <c r="I119" s="3"/>
       <c r="J119" s="7"/>
     </row>
-    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -4795,7 +4793,7 @@
       <c r="I120" s="3"/>
       <c r="J120" s="7"/>
     </row>
-    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -4823,7 +4821,7 @@
       <c r="I121" s="3"/>
       <c r="J121" s="7"/>
     </row>
-    <row r="122" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -4851,7 +4849,7 @@
       <c r="I122" s="3"/>
       <c r="J122" s="7"/>
     </row>
-    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -4879,7 +4877,7 @@
       <c r="I123" s="3"/>
       <c r="J123" s="7"/>
     </row>
-    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -4907,7 +4905,7 @@
       <c r="I124" s="3"/>
       <c r="J124" s="7"/>
     </row>
-    <row r="125" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -4935,7 +4933,7 @@
       <c r="I125" s="3"/>
       <c r="J125" s="7"/>
     </row>
-    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -4963,7 +4961,7 @@
       <c r="I126" s="3"/>
       <c r="J126" s="7"/>
     </row>
-    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -4991,7 +4989,7 @@
       <c r="I127" s="3"/>
       <c r="J127" s="7"/>
     </row>
-    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -5019,7 +5017,7 @@
       <c r="I128" s="3"/>
       <c r="J128" s="7"/>
     </row>
-    <row r="129" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -5047,7 +5045,7 @@
       <c r="I129" s="3"/>
       <c r="J129" s="7"/>
     </row>
-    <row r="130" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -5075,7 +5073,7 @@
       <c r="I130" s="3"/>
       <c r="J130" s="7"/>
     </row>
-    <row r="131" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:10" ht="27" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -5104,13 +5102,7 @@
       <c r="J131" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J131" xr:uid="{00000000-0009-0000-0000-000000000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="Easy"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A1:J131" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H2:H131" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done,Skipped"</formula1>
@@ -5118,136 +5110,136 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="E2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="E3" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="E4" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="E5" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="E6" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="E7" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="E8" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="E9" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="E10" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="E11" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="E12" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="E13" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="E14" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="E15" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
-    <hyperlink ref="E16" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="E17" r:id="rId16" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="E18" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="E19" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="E20" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="E21" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="E22" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="E23" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="E24" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="E25" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="E26" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="E27" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="E28" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="E29" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="E30" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="E31" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="E32" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="E33" r:id="rId32" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="E34" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="E35" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="E36" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="E37" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="E38" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="E39" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="E40" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="E41" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="E42" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="E43" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="E44" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="E45" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="E46" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="E47" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="E48" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="E49" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="E50" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="E51" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="E52" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="E53" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="E54" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="E55" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="E56" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="E57" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="E58" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="E59" r:id="rId58" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="E60" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="E61" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="E62" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="E63" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="E64" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="E65" r:id="rId64" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="E66" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="E67" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="E68" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="E69" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
-    <hyperlink ref="E70" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="E71" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="E72" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="E73" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="E74" r:id="rId73" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="E75" r:id="rId74" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="E76" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="E77" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="E78" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="E79" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="E80" r:id="rId79" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="E81" r:id="rId80" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="E82" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="E83" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="E84" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="E85" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="E86" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="E87" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="E88" r:id="rId87" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
-    <hyperlink ref="E89" r:id="rId88" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
-    <hyperlink ref="E90" r:id="rId89" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
-    <hyperlink ref="E91" r:id="rId90" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
-    <hyperlink ref="E92" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
-    <hyperlink ref="E93" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
-    <hyperlink ref="E94" r:id="rId93" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
-    <hyperlink ref="E95" r:id="rId94" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
-    <hyperlink ref="E96" r:id="rId95" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
-    <hyperlink ref="E97" r:id="rId96" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
-    <hyperlink ref="E98" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
-    <hyperlink ref="E99" r:id="rId98" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
-    <hyperlink ref="E100" r:id="rId99" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
-    <hyperlink ref="E101" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
-    <hyperlink ref="E102" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
-    <hyperlink ref="E103" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
-    <hyperlink ref="E104" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
-    <hyperlink ref="E105" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
-    <hyperlink ref="E106" r:id="rId105" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
-    <hyperlink ref="E107" r:id="rId106" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
-    <hyperlink ref="E108" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
-    <hyperlink ref="E109" r:id="rId108" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
-    <hyperlink ref="E110" r:id="rId109" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
-    <hyperlink ref="E111" r:id="rId110" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
-    <hyperlink ref="E112" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
-    <hyperlink ref="E113" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
-    <hyperlink ref="E114" r:id="rId113" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
-    <hyperlink ref="E115" r:id="rId114" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
-    <hyperlink ref="E116" r:id="rId115" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
-    <hyperlink ref="E117" r:id="rId116" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
-    <hyperlink ref="E118" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
-    <hyperlink ref="E119" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
-    <hyperlink ref="E120" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
-    <hyperlink ref="E121" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
-    <hyperlink ref="E122" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
-    <hyperlink ref="E123" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
-    <hyperlink ref="E124" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
-    <hyperlink ref="E125" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
-    <hyperlink ref="E126" r:id="rId125" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
-    <hyperlink ref="E127" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
-    <hyperlink ref="E128" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
-    <hyperlink ref="E129" r:id="rId128" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
-    <hyperlink ref="E130" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
-    <hyperlink ref="E131" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="E5" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
+    <hyperlink ref="E6" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
+    <hyperlink ref="E7" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
+    <hyperlink ref="E8" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
+    <hyperlink ref="E9" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
+    <hyperlink ref="E10" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
+    <hyperlink ref="E11" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
+    <hyperlink ref="E12" r:id="rId8" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
+    <hyperlink ref="E13" r:id="rId9" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
+    <hyperlink ref="E14" r:id="rId10" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
+    <hyperlink ref="E17" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
+    <hyperlink ref="E18" r:id="rId12" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
+    <hyperlink ref="E19" r:id="rId13" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
+    <hyperlink ref="E21" r:id="rId14" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
+    <hyperlink ref="E22" r:id="rId15" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
+    <hyperlink ref="E23" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
+    <hyperlink ref="E24" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
+    <hyperlink ref="E25" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
+    <hyperlink ref="E26" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
+    <hyperlink ref="E27" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
+    <hyperlink ref="E29" r:id="rId21" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
+    <hyperlink ref="E30" r:id="rId22" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
+    <hyperlink ref="E31" r:id="rId23" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
+    <hyperlink ref="E32" r:id="rId24" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
+    <hyperlink ref="E39" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
+    <hyperlink ref="E40" r:id="rId26" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
+    <hyperlink ref="E42" r:id="rId27" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
+    <hyperlink ref="E43" r:id="rId28" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="E50" r:id="rId29" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="E51" r:id="rId30" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="E52" r:id="rId31" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="E53" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="E54" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
+    <hyperlink ref="E57" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
+    <hyperlink ref="E58" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
+    <hyperlink ref="E60" r:id="rId36" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
+    <hyperlink ref="E61" r:id="rId37" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
+    <hyperlink ref="E65" r:id="rId38" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
+    <hyperlink ref="E66" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
+    <hyperlink ref="E67" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
+    <hyperlink ref="E68" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
+    <hyperlink ref="E69" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000043000000}"/>
+    <hyperlink ref="E74" r:id="rId43" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
+    <hyperlink ref="E78" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
+    <hyperlink ref="E79" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
+    <hyperlink ref="E80" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
+    <hyperlink ref="E81" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
+    <hyperlink ref="E82" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
+    <hyperlink ref="E84" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
+    <hyperlink ref="E85" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
+    <hyperlink ref="E86" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
+    <hyperlink ref="E87" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
+    <hyperlink ref="E88" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000056000000}"/>
+    <hyperlink ref="E89" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000057000000}"/>
+    <hyperlink ref="E90" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000058000000}"/>
+    <hyperlink ref="E91" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000059000000}"/>
+    <hyperlink ref="E92" r:id="rId57" xr:uid="{00000000-0004-0000-0000-00005A000000}"/>
+    <hyperlink ref="E93" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00005B000000}"/>
+    <hyperlink ref="E94" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00005C000000}"/>
+    <hyperlink ref="E95" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00005D000000}"/>
+    <hyperlink ref="E96" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00005E000000}"/>
+    <hyperlink ref="E97" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00005F000000}"/>
+    <hyperlink ref="E98" r:id="rId63" xr:uid="{00000000-0004-0000-0000-000060000000}"/>
+    <hyperlink ref="E99" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000061000000}"/>
+    <hyperlink ref="E101" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000063000000}"/>
+    <hyperlink ref="E102" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000064000000}"/>
+    <hyperlink ref="E103" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000065000000}"/>
+    <hyperlink ref="E104" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000066000000}"/>
+    <hyperlink ref="E105" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000067000000}"/>
+    <hyperlink ref="E106" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000068000000}"/>
+    <hyperlink ref="E107" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000069000000}"/>
+    <hyperlink ref="E108" r:id="rId72" xr:uid="{00000000-0004-0000-0000-00006A000000}"/>
+    <hyperlink ref="E109" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00006B000000}"/>
+    <hyperlink ref="E110" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00006C000000}"/>
+    <hyperlink ref="E111" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00006D000000}"/>
+    <hyperlink ref="E112" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00006E000000}"/>
+    <hyperlink ref="E113" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00006F000000}"/>
+    <hyperlink ref="E114" r:id="rId78" xr:uid="{00000000-0004-0000-0000-000070000000}"/>
+    <hyperlink ref="E115" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000071000000}"/>
+    <hyperlink ref="E116" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000072000000}"/>
+    <hyperlink ref="E117" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000073000000}"/>
+    <hyperlink ref="E118" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000074000000}"/>
+    <hyperlink ref="E120" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
+    <hyperlink ref="E121" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
+    <hyperlink ref="E122" r:id="rId85" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
+    <hyperlink ref="E123" r:id="rId86" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="E124" r:id="rId87" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="E125" r:id="rId88" xr:uid="{00000000-0004-0000-0000-00007B000000}"/>
+    <hyperlink ref="E126" r:id="rId89" xr:uid="{00000000-0004-0000-0000-00007C000000}"/>
+    <hyperlink ref="E127" r:id="rId90" xr:uid="{00000000-0004-0000-0000-00007D000000}"/>
+    <hyperlink ref="E128" r:id="rId91" xr:uid="{00000000-0004-0000-0000-00007E000000}"/>
+    <hyperlink ref="E129" r:id="rId92" xr:uid="{00000000-0004-0000-0000-00007F000000}"/>
+    <hyperlink ref="E130" r:id="rId93" xr:uid="{00000000-0004-0000-0000-000080000000}"/>
+    <hyperlink ref="E131" r:id="rId94" xr:uid="{00000000-0004-0000-0000-000081000000}"/>
+    <hyperlink ref="E119" r:id="rId95" xr:uid="{00000000-0004-0000-0000-000075000000}"/>
+    <hyperlink ref="E100" r:id="rId96" xr:uid="{00000000-0004-0000-0000-000062000000}"/>
+    <hyperlink ref="E83" r:id="rId97" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
+    <hyperlink ref="E77" r:id="rId98" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
+    <hyperlink ref="E76" r:id="rId99" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
+    <hyperlink ref="E75" r:id="rId100" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
+    <hyperlink ref="E73" r:id="rId101" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
+    <hyperlink ref="E72" r:id="rId102" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
+    <hyperlink ref="E71" r:id="rId103" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
+    <hyperlink ref="E70" r:id="rId104" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
+    <hyperlink ref="E64" r:id="rId105" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
+    <hyperlink ref="E63" r:id="rId106" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
+    <hyperlink ref="E62" r:id="rId107" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
+    <hyperlink ref="E59" r:id="rId108" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
+    <hyperlink ref="E56" r:id="rId109" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
+    <hyperlink ref="E55" r:id="rId110" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
+    <hyperlink ref="E49" r:id="rId111" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="E48" r:id="rId112" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="E47" r:id="rId113" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="E46" r:id="rId114" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="E45" r:id="rId115" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="E44" r:id="rId116" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="E41" r:id="rId117" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
+    <hyperlink ref="E38" r:id="rId118" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
+    <hyperlink ref="E37" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
+    <hyperlink ref="E36" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
+    <hyperlink ref="E35" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
+    <hyperlink ref="E34" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
+    <hyperlink ref="E33" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
+    <hyperlink ref="E28" r:id="rId124" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
+    <hyperlink ref="E20" r:id="rId125" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
+    <hyperlink ref="E16" r:id="rId126" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
+    <hyperlink ref="E15" r:id="rId127" xr:uid="{00000000-0004-0000-0000-00000D000000}"/>
+    <hyperlink ref="E4" r:id="rId128" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
+    <hyperlink ref="E3" r:id="rId129" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
+    <hyperlink ref="E2" r:id="rId130" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -5322,7 +5314,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF('130-Day Plan'!H2:H131,"Not Started")</f>
-        <v>121</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>

<commit_message>
day 14 2 pgms
</commit_message>
<xml_diff>
--- a/3aed9d04-2385-4fdd-b403-316e5db325c7.xlsx
+++ b/3aed9d04-2385-4fdd-b403-316e5db325c7.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Desktop\DSA\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A368371-1742-4245-9943-C5D902F52B6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E93E71E-2D96-4BC8-913D-D374D6061907}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="11625" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1414,6 +1414,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:J131"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
@@ -1461,7 +1462,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -1489,7 +1490,7 @@
       <c r="I2" s="3"/>
       <c r="J2" s="7"/>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -1517,7 +1518,7 @@
       <c r="I3" s="3"/>
       <c r="J3" s="7"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -1545,7 +1546,7 @@
       <c r="I4" s="3"/>
       <c r="J4" s="7"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -1573,7 +1574,7 @@
       <c r="I5" s="3"/>
       <c r="J5" s="7"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -1601,7 +1602,7 @@
       <c r="I6" s="3"/>
       <c r="J6" s="7"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -1629,7 +1630,7 @@
       <c r="I7" s="3"/>
       <c r="J7" s="7"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -1657,7 +1658,7 @@
       <c r="I8" s="3"/>
       <c r="J8" s="7"/>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A9" s="2">
         <v>8</v>
       </c>
@@ -1685,7 +1686,7 @@
       <c r="I9" s="3"/>
       <c r="J9" s="7"/>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -1713,7 +1714,7 @@
       <c r="I10" s="3"/>
       <c r="J10" s="7"/>
     </row>
-    <row r="11" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A11" s="2">
         <v>10</v>
       </c>
@@ -1741,7 +1742,7 @@
       <c r="I11" s="3"/>
       <c r="J11" s="7"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A12" s="2">
         <v>11</v>
       </c>
@@ -1769,7 +1770,7 @@
       <c r="I12" s="3"/>
       <c r="J12" s="7"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A13" s="2">
         <v>12</v>
       </c>
@@ -1797,7 +1798,7 @@
       <c r="I13" s="3"/>
       <c r="J13" s="7"/>
     </row>
-    <row r="14" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A14" s="2">
         <v>13</v>
       </c>
@@ -1825,7 +1826,7 @@
       <c r="I14" s="3"/>
       <c r="J14" s="7"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A15" s="2">
         <v>14</v>
       </c>
@@ -1848,12 +1849,12 @@
         <v>43</v>
       </c>
       <c r="H15" s="7" t="s">
-        <v>15</v>
+        <v>302</v>
       </c>
       <c r="I15" s="3"/>
       <c r="J15" s="7"/>
     </row>
-    <row r="16" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A16" s="2">
         <v>15</v>
       </c>
@@ -1876,12 +1877,12 @@
         <v>45</v>
       </c>
       <c r="H16" s="7" t="s">
-        <v>15</v>
+        <v>302</v>
       </c>
       <c r="I16" s="3"/>
       <c r="J16" s="7"/>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A17" s="2">
         <v>16</v>
       </c>
@@ -1904,12 +1905,12 @@
         <v>47</v>
       </c>
       <c r="H17" s="7" t="s">
-        <v>15</v>
+        <v>303</v>
       </c>
       <c r="I17" s="3"/>
       <c r="J17" s="7"/>
     </row>
-    <row r="18" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A18" s="2">
         <v>17</v>
       </c>
@@ -1937,7 +1938,7 @@
       <c r="I18" s="3"/>
       <c r="J18" s="7"/>
     </row>
-    <row r="19" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A19" s="2">
         <v>18</v>
       </c>
@@ -1993,7 +1994,7 @@
       <c r="I20" s="3"/>
       <c r="J20" s="7"/>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A21" s="2">
         <v>20</v>
       </c>
@@ -2021,7 +2022,7 @@
       <c r="I21" s="3"/>
       <c r="J21" s="7"/>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A22" s="2">
         <v>21</v>
       </c>
@@ -2049,7 +2050,7 @@
       <c r="I22" s="3"/>
       <c r="J22" s="7"/>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A23" s="2">
         <v>22</v>
       </c>
@@ -2077,7 +2078,7 @@
       <c r="I23" s="3"/>
       <c r="J23" s="7"/>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A24" s="2">
         <v>23</v>
       </c>
@@ -2105,7 +2106,7 @@
       <c r="I24" s="3"/>
       <c r="J24" s="7"/>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A25" s="2">
         <v>24</v>
       </c>
@@ -2133,7 +2134,7 @@
       <c r="I25" s="3"/>
       <c r="J25" s="7"/>
     </row>
-    <row r="26" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A26" s="2">
         <v>25</v>
       </c>
@@ -2161,7 +2162,7 @@
       <c r="I26" s="3"/>
       <c r="J26" s="7"/>
     </row>
-    <row r="27" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A27" s="2">
         <v>26</v>
       </c>
@@ -2217,7 +2218,7 @@
       <c r="I28" s="3"/>
       <c r="J28" s="7"/>
     </row>
-    <row r="29" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A29" s="2">
         <v>28</v>
       </c>
@@ -2245,7 +2246,7 @@
       <c r="I29" s="3"/>
       <c r="J29" s="7"/>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A30" s="2">
         <v>29</v>
       </c>
@@ -2273,7 +2274,7 @@
       <c r="I30" s="3"/>
       <c r="J30" s="7"/>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="31" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A31" s="2">
         <v>30</v>
       </c>
@@ -2301,7 +2302,7 @@
       <c r="I31" s="3"/>
       <c r="J31" s="7"/>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A32" s="2">
         <v>31</v>
       </c>
@@ -2497,7 +2498,7 @@
       <c r="I38" s="3"/>
       <c r="J38" s="7"/>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="39" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A39" s="2">
         <v>38</v>
       </c>
@@ -2525,7 +2526,7 @@
       <c r="I39" s="3"/>
       <c r="J39" s="7"/>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="40" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A40" s="2">
         <v>39</v>
       </c>
@@ -2581,7 +2582,7 @@
       <c r="I41" s="3"/>
       <c r="J41" s="7"/>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="42" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A42" s="2">
         <v>41</v>
       </c>
@@ -2609,7 +2610,7 @@
       <c r="I42" s="3"/>
       <c r="J42" s="7"/>
     </row>
-    <row r="43" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="43" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A43" s="2">
         <v>42</v>
       </c>
@@ -2805,7 +2806,7 @@
       <c r="I49" s="3"/>
       <c r="J49" s="7"/>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="50" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A50" s="2">
         <v>49</v>
       </c>
@@ -2833,7 +2834,7 @@
       <c r="I50" s="3"/>
       <c r="J50" s="7"/>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A51" s="2">
         <v>50</v>
       </c>
@@ -2861,7 +2862,7 @@
       <c r="I51" s="3"/>
       <c r="J51" s="7"/>
     </row>
-    <row r="52" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="52" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A52" s="2">
         <v>51</v>
       </c>
@@ -2889,7 +2890,7 @@
       <c r="I52" s="3"/>
       <c r="J52" s="7"/>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="53" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A53" s="2">
         <v>52</v>
       </c>
@@ -2917,7 +2918,7 @@
       <c r="I53" s="3"/>
       <c r="J53" s="7"/>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="54" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A54" s="2">
         <v>53</v>
       </c>
@@ -3001,7 +3002,7 @@
       <c r="I56" s="3"/>
       <c r="J56" s="7"/>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="57" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A57" s="2">
         <v>56</v>
       </c>
@@ -3029,7 +3030,7 @@
       <c r="I57" s="3"/>
       <c r="J57" s="7"/>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="58" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A58" s="2">
         <v>57</v>
       </c>
@@ -3085,7 +3086,7 @@
       <c r="I59" s="3"/>
       <c r="J59" s="7"/>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="60" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A60" s="2">
         <v>59</v>
       </c>
@@ -3113,7 +3114,7 @@
       <c r="I60" s="3"/>
       <c r="J60" s="7"/>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="61" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A61" s="2">
         <v>60</v>
       </c>
@@ -3225,7 +3226,7 @@
       <c r="I64" s="3"/>
       <c r="J64" s="7"/>
     </row>
-    <row r="65" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="65" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A65" s="2">
         <v>64</v>
       </c>
@@ -3253,7 +3254,7 @@
       <c r="I65" s="3"/>
       <c r="J65" s="7"/>
     </row>
-    <row r="66" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="66" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A66" s="2">
         <v>65</v>
       </c>
@@ -3281,7 +3282,7 @@
       <c r="I66" s="3"/>
       <c r="J66" s="7"/>
     </row>
-    <row r="67" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="67" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A67" s="2">
         <v>66</v>
       </c>
@@ -3309,7 +3310,7 @@
       <c r="I67" s="3"/>
       <c r="J67" s="7"/>
     </row>
-    <row r="68" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="68" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A68" s="2">
         <v>67</v>
       </c>
@@ -3337,7 +3338,7 @@
       <c r="I68" s="3"/>
       <c r="J68" s="7"/>
     </row>
-    <row r="69" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="69" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A69" s="2">
         <v>68</v>
       </c>
@@ -3477,7 +3478,7 @@
       <c r="I73" s="3"/>
       <c r="J73" s="7"/>
     </row>
-    <row r="74" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="74" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A74" s="2">
         <v>73</v>
       </c>
@@ -3589,7 +3590,7 @@
       <c r="I77" s="3"/>
       <c r="J77" s="7"/>
     </row>
-    <row r="78" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="78" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A78" s="2">
         <v>77</v>
       </c>
@@ -3617,7 +3618,7 @@
       <c r="I78" s="3"/>
       <c r="J78" s="7"/>
     </row>
-    <row r="79" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="79" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A79" s="2">
         <v>78</v>
       </c>
@@ -3645,7 +3646,7 @@
       <c r="I79" s="3"/>
       <c r="J79" s="7"/>
     </row>
-    <row r="80" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="80" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A80" s="2">
         <v>79</v>
       </c>
@@ -3673,7 +3674,7 @@
       <c r="I80" s="3"/>
       <c r="J80" s="7"/>
     </row>
-    <row r="81" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="81" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A81" s="2">
         <v>80</v>
       </c>
@@ -3701,7 +3702,7 @@
       <c r="I81" s="3"/>
       <c r="J81" s="7"/>
     </row>
-    <row r="82" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="82" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A82" s="2">
         <v>81</v>
       </c>
@@ -3757,7 +3758,7 @@
       <c r="I83" s="3"/>
       <c r="J83" s="7"/>
     </row>
-    <row r="84" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="84" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A84" s="2">
         <v>83</v>
       </c>
@@ -3785,7 +3786,7 @@
       <c r="I84" s="3"/>
       <c r="J84" s="7"/>
     </row>
-    <row r="85" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="85" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A85" s="2">
         <v>84</v>
       </c>
@@ -3813,7 +3814,7 @@
       <c r="I85" s="3"/>
       <c r="J85" s="7"/>
     </row>
-    <row r="86" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="86" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A86" s="2">
         <v>85</v>
       </c>
@@ -3841,7 +3842,7 @@
       <c r="I86" s="3"/>
       <c r="J86" s="7"/>
     </row>
-    <row r="87" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="87" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A87" s="2">
         <v>86</v>
       </c>
@@ -3869,7 +3870,7 @@
       <c r="I87" s="3"/>
       <c r="J87" s="7"/>
     </row>
-    <row r="88" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="88" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A88" s="2">
         <v>87</v>
       </c>
@@ -3897,7 +3898,7 @@
       <c r="I88" s="3"/>
       <c r="J88" s="7"/>
     </row>
-    <row r="89" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="89" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A89" s="2">
         <v>88</v>
       </c>
@@ -3925,7 +3926,7 @@
       <c r="I89" s="3"/>
       <c r="J89" s="7"/>
     </row>
-    <row r="90" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="90" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A90" s="2">
         <v>89</v>
       </c>
@@ -3953,7 +3954,7 @@
       <c r="I90" s="3"/>
       <c r="J90" s="7"/>
     </row>
-    <row r="91" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="91" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A91" s="2">
         <v>90</v>
       </c>
@@ -3981,7 +3982,7 @@
       <c r="I91" s="3"/>
       <c r="J91" s="7"/>
     </row>
-    <row r="92" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="92" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A92" s="2">
         <v>91</v>
       </c>
@@ -4009,7 +4010,7 @@
       <c r="I92" s="3"/>
       <c r="J92" s="7"/>
     </row>
-    <row r="93" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="93" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A93" s="2">
         <v>92</v>
       </c>
@@ -4037,7 +4038,7 @@
       <c r="I93" s="3"/>
       <c r="J93" s="7"/>
     </row>
-    <row r="94" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="94" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A94" s="2">
         <v>93</v>
       </c>
@@ -4065,7 +4066,7 @@
       <c r="I94" s="3"/>
       <c r="J94" s="7"/>
     </row>
-    <row r="95" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="95" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A95" s="2">
         <v>94</v>
       </c>
@@ -4093,7 +4094,7 @@
       <c r="I95" s="3"/>
       <c r="J95" s="7"/>
     </row>
-    <row r="96" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="96" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A96" s="2">
         <v>95</v>
       </c>
@@ -4121,7 +4122,7 @@
       <c r="I96" s="3"/>
       <c r="J96" s="7"/>
     </row>
-    <row r="97" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="97" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A97" s="2">
         <v>96</v>
       </c>
@@ -4149,7 +4150,7 @@
       <c r="I97" s="3"/>
       <c r="J97" s="7"/>
     </row>
-    <row r="98" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="98" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A98" s="2">
         <v>97</v>
       </c>
@@ -4177,7 +4178,7 @@
       <c r="I98" s="3"/>
       <c r="J98" s="7"/>
     </row>
-    <row r="99" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="99" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A99" s="2">
         <v>98</v>
       </c>
@@ -4233,7 +4234,7 @@
       <c r="I100" s="3"/>
       <c r="J100" s="7"/>
     </row>
-    <row r="101" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="101" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A101" s="2">
         <v>100</v>
       </c>
@@ -4261,7 +4262,7 @@
       <c r="I101" s="3"/>
       <c r="J101" s="7"/>
     </row>
-    <row r="102" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="102" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A102" s="2">
         <v>101</v>
       </c>
@@ -4289,7 +4290,7 @@
       <c r="I102" s="3"/>
       <c r="J102" s="7"/>
     </row>
-    <row r="103" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="103" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A103" s="2">
         <v>102</v>
       </c>
@@ -4317,7 +4318,7 @@
       <c r="I103" s="3"/>
       <c r="J103" s="7"/>
     </row>
-    <row r="104" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="104" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A104" s="2">
         <v>103</v>
       </c>
@@ -4345,7 +4346,7 @@
       <c r="I104" s="3"/>
       <c r="J104" s="7"/>
     </row>
-    <row r="105" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="105" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A105" s="2">
         <v>104</v>
       </c>
@@ -4373,7 +4374,7 @@
       <c r="I105" s="3"/>
       <c r="J105" s="7"/>
     </row>
-    <row r="106" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="106" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A106" s="2">
         <v>105</v>
       </c>
@@ -4401,7 +4402,7 @@
       <c r="I106" s="3"/>
       <c r="J106" s="7"/>
     </row>
-    <row r="107" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="107" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A107" s="2">
         <v>106</v>
       </c>
@@ -4429,7 +4430,7 @@
       <c r="I107" s="3"/>
       <c r="J107" s="7"/>
     </row>
-    <row r="108" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="108" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A108" s="2">
         <v>107</v>
       </c>
@@ -4457,7 +4458,7 @@
       <c r="I108" s="3"/>
       <c r="J108" s="7"/>
     </row>
-    <row r="109" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="109" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A109" s="2">
         <v>108</v>
       </c>
@@ -4485,7 +4486,7 @@
       <c r="I109" s="3"/>
       <c r="J109" s="7"/>
     </row>
-    <row r="110" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="110" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A110" s="2">
         <v>109</v>
       </c>
@@ -4513,7 +4514,7 @@
       <c r="I110" s="3"/>
       <c r="J110" s="7"/>
     </row>
-    <row r="111" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="111" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A111" s="2">
         <v>110</v>
       </c>
@@ -4541,7 +4542,7 @@
       <c r="I111" s="3"/>
       <c r="J111" s="7"/>
     </row>
-    <row r="112" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="112" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A112" s="2">
         <v>111</v>
       </c>
@@ -4569,7 +4570,7 @@
       <c r="I112" s="3"/>
       <c r="J112" s="7"/>
     </row>
-    <row r="113" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="113" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A113" s="2">
         <v>112</v>
       </c>
@@ -4597,7 +4598,7 @@
       <c r="I113" s="3"/>
       <c r="J113" s="7"/>
     </row>
-    <row r="114" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="114" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A114" s="2">
         <v>113</v>
       </c>
@@ -4625,7 +4626,7 @@
       <c r="I114" s="3"/>
       <c r="J114" s="7"/>
     </row>
-    <row r="115" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="115" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A115" s="2">
         <v>114</v>
       </c>
@@ -4653,7 +4654,7 @@
       <c r="I115" s="3"/>
       <c r="J115" s="7"/>
     </row>
-    <row r="116" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="116" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A116" s="2">
         <v>115</v>
       </c>
@@ -4681,7 +4682,7 @@
       <c r="I116" s="3"/>
       <c r="J116" s="7"/>
     </row>
-    <row r="117" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="117" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A117" s="2">
         <v>116</v>
       </c>
@@ -4709,7 +4710,7 @@
       <c r="I117" s="3"/>
       <c r="J117" s="7"/>
     </row>
-    <row r="118" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="118" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A118" s="2">
         <v>117</v>
       </c>
@@ -4765,7 +4766,7 @@
       <c r="I119" s="3"/>
       <c r="J119" s="7"/>
     </row>
-    <row r="120" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="120" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A120" s="2">
         <v>119</v>
       </c>
@@ -4793,7 +4794,7 @@
       <c r="I120" s="3"/>
       <c r="J120" s="7"/>
     </row>
-    <row r="121" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="121" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A121" s="2">
         <v>120</v>
       </c>
@@ -4821,7 +4822,7 @@
       <c r="I121" s="3"/>
       <c r="J121" s="7"/>
     </row>
-    <row r="122" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="122" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A122" s="2">
         <v>121</v>
       </c>
@@ -4849,7 +4850,7 @@
       <c r="I122" s="3"/>
       <c r="J122" s="7"/>
     </row>
-    <row r="123" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="123" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A123" s="2">
         <v>122</v>
       </c>
@@ -4877,7 +4878,7 @@
       <c r="I123" s="3"/>
       <c r="J123" s="7"/>
     </row>
-    <row r="124" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="124" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A124" s="2">
         <v>123</v>
       </c>
@@ -4905,7 +4906,7 @@
       <c r="I124" s="3"/>
       <c r="J124" s="7"/>
     </row>
-    <row r="125" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="125" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A125" s="2">
         <v>124</v>
       </c>
@@ -4933,7 +4934,7 @@
       <c r="I125" s="3"/>
       <c r="J125" s="7"/>
     </row>
-    <row r="126" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="126" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A126" s="2">
         <v>125</v>
       </c>
@@ -4961,7 +4962,7 @@
       <c r="I126" s="3"/>
       <c r="J126" s="7"/>
     </row>
-    <row r="127" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="127" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A127" s="2">
         <v>126</v>
       </c>
@@ -4989,7 +4990,7 @@
       <c r="I127" s="3"/>
       <c r="J127" s="7"/>
     </row>
-    <row r="128" spans="1:10" x14ac:dyDescent="0.45">
+    <row r="128" spans="1:10" hidden="1" x14ac:dyDescent="0.45">
       <c r="A128" s="2">
         <v>127</v>
       </c>
@@ -5017,7 +5018,7 @@
       <c r="I128" s="3"/>
       <c r="J128" s="7"/>
     </row>
-    <row r="129" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="129" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A129" s="2">
         <v>128</v>
       </c>
@@ -5045,7 +5046,7 @@
       <c r="I129" s="3"/>
       <c r="J129" s="7"/>
     </row>
-    <row r="130" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="130" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A130" s="2">
         <v>129</v>
       </c>
@@ -5073,7 +5074,7 @@
       <c r="I130" s="3"/>
       <c r="J130" s="7"/>
     </row>
-    <row r="131" spans="1:10" ht="27" x14ac:dyDescent="0.45">
+    <row r="131" spans="1:10" ht="27" hidden="1" x14ac:dyDescent="0.45">
       <c r="A131" s="2">
         <v>130</v>
       </c>
@@ -5102,7 +5103,18 @@
       <c r="J131" s="7"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J131" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:J131" xr:uid="{00000000-0009-0000-0000-000000000000}">
+    <filterColumn colId="3">
+      <filters>
+        <filter val="Easy"/>
+      </filters>
+    </filterColumn>
+    <filterColumn colId="7">
+      <filters>
+        <filter val="Not Started"/>
+      </filters>
+    </filterColumn>
+  </autoFilter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" sqref="H2:H131" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"Not Started,In Progress,Done,Skipped"</formula1>
@@ -5314,7 +5326,7 @@
       </c>
       <c r="B6" s="12">
         <f>COUNTIF('130-Day Plan'!H2:H131,"Not Started")</f>
-        <v>118</v>
+        <v>115</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">

</xml_diff>